<commit_message>
chore: remove scratch directory and update project files
</commit_message>
<xml_diff>
--- a/database/temp.xlsx
+++ b/database/temp.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\User Vinatech.DESKTOP-RJJSEQU\Desktop\database\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="8_{A1656CF7-EAF6-403C-A7C1-7FA282BA65E0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{0B13E81E-6B91-43C6-ABC0-B499E757A061}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{3A47A83A-EDBF-491B-87BA-CC4E501F318B}"/>
   </bookViews>
@@ -1105,7 +1105,7 @@
     <col min="31" max="31" width="13.5546875" bestFit="1" customWidth="1"/>
     <col min="32" max="32" width="13.21875" bestFit="1" customWidth="1"/>
     <col min="33" max="33" width="15.33203125" bestFit="1" customWidth="1"/>
-    <col min="34" max="34" width="13.6640625" bestFit="1" customWidth="1"/>
+    <col min="34" max="34" width="14.6640625" bestFit="1" customWidth="1"/>
     <col min="35" max="35" width="20.33203125" bestFit="1" customWidth="1"/>
     <col min="36" max="39" width="10.109375" bestFit="1" customWidth="1"/>
     <col min="40" max="40" width="9" bestFit="1" customWidth="1"/>

</xml_diff>